<commit_message>
Pinkerton and Possessions fix
</commit_message>
<xml_diff>
--- a/Div_Roads Project.xlsx
+++ b/Div_Roads Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b94b8e39c9d805aa/Documents/GitHub/Diverging-Roads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="152" documentId="11_F25DC773A252ABDACC10484719DA7CD85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBABFD3E-7549-41E3-BE61-8CA24F01C92A}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="11_F25DC773A252ABDACC10484719DA7CD85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A673732B-858A-40E5-8E49-980F4A0D5C0B}"/>
   <bookViews>
-    <workbookView xWindow="225" yWindow="825" windowWidth="17655" windowHeight="12660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1365" yWindow="165" windowWidth="17655" windowHeight="12660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="49">
   <si>
     <t>Title</t>
   </si>
@@ -153,10 +153,25 @@
     <t>Copyright added</t>
   </si>
   <si>
-    <t>Need to fix mansion image width</t>
-  </si>
-  <si>
     <t>Text in original and lebtown differ - reconcile</t>
+  </si>
+  <si>
+    <t>Check why the "topic tag" on the index.html listing</t>
+  </si>
+  <si>
+    <t>Done, defined the small and medium plate sizes in readme file.</t>
+  </si>
+  <si>
+    <t>Check iPad format</t>
+  </si>
+  <si>
+    <t>Create Word Doc</t>
+  </si>
+  <si>
+    <t>Clean out "Who Knew" folder</t>
+  </si>
+  <si>
+    <t>Forced to fit, but need a generic external stylesheet solution</t>
   </si>
 </sst>
 </file>
@@ -181,12 +196,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -201,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -215,14 +242,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -508,54 +538,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="7.28515625" style="2" customWidth="1"/>
     <col min="4" max="4" width="8.5703125" style="2" customWidth="1"/>
     <col min="5" max="5" width="10.5703125" style="4" customWidth="1"/>
     <col min="6" max="6" width="9.85546875" style="3" customWidth="1"/>
     <col min="7" max="7" width="10" style="3" customWidth="1"/>
     <col min="8" max="8" width="25.85546875" style="1" customWidth="1"/>
     <col min="9" max="9" width="19.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="5"/>
+    <col min="10" max="10" width="9.140625" style="3"/>
+    <col min="13" max="13" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="6" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:14" s="5" customFormat="1" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="6" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="N1" s="6"/>
+    </row>
+    <row r="2" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -583,11 +624,11 @@
       <c r="I2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="J2" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -612,14 +653,14 @@
       <c r="H3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -632,8 +673,23 @@
       <c r="E4" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -647,7 +703,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -661,7 +717,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -675,7 +731,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -689,7 +745,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -703,7 +759,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -717,7 +773,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -731,7 +787,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -745,7 +801,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -759,7 +815,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -773,7 +829,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -787,7 +843,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -801,7 +857,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -815,7 +871,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -829,7 +885,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -843,7 +899,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -857,7 +913,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -871,7 +927,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -885,10 +941,10 @@
         <v>33</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -901,8 +957,11 @@
       <c r="E23" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J23" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -910,7 +969,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -921,7 +980,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -932,7 +991,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -943,7 +1002,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -954,7 +1013,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -965,12 +1024,12 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>

</xml_diff>